<commit_message>
File tính giá: tự tra cước VPS và AM đi US; Prompt Nhập hàng thu cân nặng, kích thước, số lượng
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tzo4cxCWwqApfnWJKtieJn
</commit_message>
<xml_diff>
--- a/files/TinhGia_TuDong.xlsx
+++ b/files/TinhGia_TuDong.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DỮ LIỆU FASTMOSS" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NHẬP HÀNG" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KẾT QUẢ" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CƯỚC VẬN CHUYỂN" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -57,7 +58,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +78,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -118,6 +124,7 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -126,12 +133,19 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -705,23 +719,55 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Tỷ giá VND sang USD (dùng đổi cước vận chuyển)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>26000</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Cập nhật theo tỷ giá hiện tại</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Hãng vận chuyển đi US (Rẻ nhất, VPS hoặc AM)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Rẻ nhất</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Chỉ dùng khi bán US</t>
+        </is>
+      </c>
+    </row>
     <row r="15" ht="44" customHeight="1">
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Phí sàn</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>VN (VND)</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>US (USD)</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
@@ -739,7 +785,7 @@
       <c r="D16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>VN: kiểm tra Seller Center. US: giá trị mẫu, nhập lại theo sàn.</t>
         </is>
@@ -757,7 +803,7 @@
       <c r="D17" s="6" t="n">
         <v>0.06</v>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>Thay bằng mức của ngành bạn bán.</t>
         </is>
@@ -775,7 +821,7 @@
       <c r="D18" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Giá trị mẫu.</t>
         </is>
@@ -793,7 +839,7 @@
       <c r="D19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>VN: thuế hộ kinh doanh. US: giá trị mẫu.</t>
         </is>
@@ -807,7 +853,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Rẻ nhất,VPS,AM"</formula1>
+    </dataValidation>
     <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VN,US"</formula1>
     </dataValidation>
@@ -856,236 +905,236 @@
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Mã SP</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Loại</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Tên sản phẩm</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Giá thấp nhất</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Giá trung vị</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Giá cao nhất</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>Giá shop bán chạy nhất</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>Tổng số bán 28 ngày</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="10" t="inlineStr">
         <is>
           <t>Hoa hồng affiliate (số %, ví dụ 10)</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="10" t="inlineStr">
         <is>
           <t>% GMV từ affiliate</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>% GMV từ quảng cáo</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="L4" s="10" t="inlineStr">
         <is>
           <t>Số đối thủ</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="M4" s="10" t="inlineStr">
         <is>
           <t>Nhận định thị trường</t>
         </is>
       </c>
-      <c r="N4" s="9" t="inlineStr">
+      <c r="N4" s="10" t="inlineStr">
         <is>
           <t>Link FastMoss</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n"/>
-      <c r="B5" s="11" t="n"/>
-      <c r="C5" s="11" t="n"/>
-      <c r="D5" s="12" t="n"/>
-      <c r="E5" s="12" t="n"/>
-      <c r="F5" s="12" t="n"/>
-      <c r="G5" s="12" t="n"/>
-      <c r="H5" s="11" t="n"/>
-      <c r="I5" s="11" t="n"/>
-      <c r="J5" s="11" t="n"/>
-      <c r="K5" s="11" t="n"/>
-      <c r="L5" s="11" t="n"/>
-      <c r="M5" s="11" t="n"/>
-      <c r="N5" s="11" t="n"/>
+      <c r="A5" s="12" t="n"/>
+      <c r="B5" s="12" t="n"/>
+      <c r="C5" s="12" t="n"/>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="13" t="n"/>
+      <c r="G5" s="13" t="n"/>
+      <c r="H5" s="12" t="n"/>
+      <c r="I5" s="12" t="n"/>
+      <c r="J5" s="12" t="n"/>
+      <c r="K5" s="12" t="n"/>
+      <c r="L5" s="12" t="n"/>
+      <c r="M5" s="12" t="n"/>
+      <c r="N5" s="12" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="12" t="n"/>
-      <c r="E6" s="12" t="n"/>
-      <c r="F6" s="12" t="n"/>
-      <c r="G6" s="12" t="n"/>
-      <c r="H6" s="11" t="n"/>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="11" t="n"/>
-      <c r="K6" s="11" t="n"/>
-      <c r="L6" s="11" t="n"/>
-      <c r="M6" s="11" t="n"/>
-      <c r="N6" s="11" t="n"/>
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="13" t="n"/>
+      <c r="F6" s="13" t="n"/>
+      <c r="G6" s="13" t="n"/>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="12" t="n"/>
+      <c r="L6" s="12" t="n"/>
+      <c r="M6" s="12" t="n"/>
+      <c r="N6" s="12" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n"/>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="12" t="n"/>
-      <c r="E7" s="12" t="n"/>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="12" t="n"/>
-      <c r="H7" s="11" t="n"/>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="11" t="n"/>
-      <c r="K7" s="11" t="n"/>
-      <c r="L7" s="11" t="n"/>
-      <c r="M7" s="11" t="n"/>
-      <c r="N7" s="11" t="n"/>
+      <c r="A7" s="12" t="n"/>
+      <c r="B7" s="12" t="n"/>
+      <c r="C7" s="12" t="n"/>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="13" t="n"/>
+      <c r="G7" s="13" t="n"/>
+      <c r="H7" s="12" t="n"/>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="12" t="n"/>
+      <c r="L7" s="12" t="n"/>
+      <c r="M7" s="12" t="n"/>
+      <c r="N7" s="12" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="11" t="n"/>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="11" t="n"/>
-      <c r="K8" s="11" t="n"/>
-      <c r="L8" s="11" t="n"/>
-      <c r="M8" s="11" t="n"/>
-      <c r="N8" s="11" t="n"/>
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="13" t="n"/>
+      <c r="E8" s="13" t="n"/>
+      <c r="F8" s="13" t="n"/>
+      <c r="G8" s="13" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="12" t="n"/>
+      <c r="L8" s="12" t="n"/>
+      <c r="M8" s="12" t="n"/>
+      <c r="N8" s="12" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="12" t="n"/>
-      <c r="H9" s="11" t="n"/>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="11" t="n"/>
-      <c r="L9" s="11" t="n"/>
-      <c r="M9" s="11" t="n"/>
-      <c r="N9" s="11" t="n"/>
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="12" t="n"/>
+      <c r="L9" s="12" t="n"/>
+      <c r="M9" s="12" t="n"/>
+      <c r="N9" s="12" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="12" t="n"/>
-      <c r="H10" s="11" t="n"/>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="11" t="n"/>
-      <c r="K10" s="11" t="n"/>
-      <c r="L10" s="11" t="n"/>
-      <c r="M10" s="11" t="n"/>
-      <c r="N10" s="11" t="n"/>
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="13" t="n"/>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="12" t="n"/>
+      <c r="L10" s="12" t="n"/>
+      <c r="M10" s="12" t="n"/>
+      <c r="N10" s="12" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="11" t="n"/>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="n"/>
-      <c r="K11" s="11" t="n"/>
-      <c r="L11" s="11" t="n"/>
-      <c r="M11" s="11" t="n"/>
-      <c r="N11" s="11" t="n"/>
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="13" t="n"/>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="12" t="n"/>
+      <c r="L11" s="12" t="n"/>
+      <c r="M11" s="12" t="n"/>
+      <c r="N11" s="12" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="n"/>
-      <c r="H12" s="11" t="n"/>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n"/>
-      <c r="K12" s="11" t="n"/>
-      <c r="L12" s="11" t="n"/>
-      <c r="M12" s="11" t="n"/>
-      <c r="N12" s="11" t="n"/>
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="12" t="n"/>
+      <c r="L12" s="12" t="n"/>
+      <c r="M12" s="12" t="n"/>
+      <c r="N12" s="12" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="12" t="n"/>
-      <c r="H13" s="11" t="n"/>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n"/>
-      <c r="L13" s="11" t="n"/>
-      <c r="M13" s="11" t="n"/>
-      <c r="N13" s="11" t="n"/>
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="12" t="n"/>
+      <c r="L13" s="12" t="n"/>
+      <c r="M13" s="12" t="n"/>
+      <c r="N13" s="12" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="12" t="n"/>
-      <c r="F14" s="12" t="n"/>
-      <c r="G14" s="12" t="n"/>
-      <c r="H14" s="11" t="n"/>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="11" t="n"/>
-      <c r="L14" s="11" t="n"/>
-      <c r="M14" s="11" t="n"/>
-      <c r="N14" s="11" t="n"/>
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="12" t="n"/>
+      <c r="L14" s="12" t="n"/>
+      <c r="M14" s="12" t="n"/>
+      <c r="N14" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1098,21 +1147,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1125,69 +1185,124 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Dán kết quả của PROMPT NHẬP HÀNG vào ô C5 (không dán tiêu đề), thứ tự dòng giống sheet DỮ LIỆU FASTMOSS. Cột A, B tự hiện.</t>
+          <t>Dán kết quả của PROMPT NHẬP HÀNG vào ô C5 (không dán tiêu đề, 14 cột C đến P), thứ tự dòng giống sheet DỮ LIỆU FASTMOSS. Cột A, B và các cột xám Q đến W tự tính.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Mã SP</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Tên sản phẩm</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Giá nhập mỗi cái</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Cân nặng mỗi cái (kg)</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>Giá ship quốc tế mỗi kg</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Dài (cm)</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Rộng (cm)</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Cao (cm)</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Số lượng nhập thử</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>Giá ship mỗi kg (trống = tự tính bảng cước US)</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
         <is>
           <t>Fulfillment mỗi đơn</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>Logistics đầu đích mỗi đơn</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="L4" s="10" t="inlineStr">
         <is>
           <t>Logistics VN mỗi đơn</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="M4" s="10" t="inlineStr">
         <is>
           <t>Packing mỗi đơn</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="N4" s="10" t="inlineStr">
         <is>
           <t>MOQ</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="O4" s="10" t="inlineStr">
         <is>
           <t>Nhà cung cấp</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="P4" s="10" t="inlineStr">
         <is>
           <t>Giá bán dự kiến (trống = dùng giá trung vị)</t>
+        </is>
+      </c>
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t>Cân nặng tính cước mỗi cái (kg)</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t>Tổng kg cả lô</t>
+        </is>
+      </c>
+      <c r="S4" s="10" t="inlineStr">
+        <is>
+          <t>Cước VPS cả lô (VND)</t>
+        </is>
+      </c>
+      <c r="T4" s="10" t="inlineStr">
+        <is>
+          <t>Cước AM cả lô (VND)</t>
+        </is>
+      </c>
+      <c r="U4" s="10" t="inlineStr">
+        <is>
+          <t>Hãng được chọn</t>
+        </is>
+      </c>
+      <c r="V4" s="10" t="inlineStr">
+        <is>
+          <t>Cước cả lô được chọn (VND)</t>
+        </is>
+      </c>
+      <c r="W4" s="10" t="inlineStr">
+        <is>
+          <t>Ship quốc tế mỗi cái</t>
         </is>
       </c>
     </row>
@@ -1200,16 +1315,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C5="","",'DỮ LIỆU FASTMOSS'!C5)</f>
         <v/>
       </c>
-      <c r="C5" s="12" t="n"/>
-      <c r="D5" s="11" t="n"/>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="12" t="n"/>
       <c r="E5" s="12" t="n"/>
       <c r="F5" s="12" t="n"/>
       <c r="G5" s="12" t="n"/>
       <c r="H5" s="12" t="n"/>
-      <c r="I5" s="12" t="n"/>
-      <c r="J5" s="11" t="n"/>
-      <c r="K5" s="11" t="n"/>
-      <c r="L5" s="12" t="n"/>
+      <c r="I5" s="13" t="n"/>
+      <c r="J5" s="13" t="n"/>
+      <c r="K5" s="13" t="n"/>
+      <c r="L5" s="13" t="n"/>
+      <c r="M5" s="13" t="n"/>
+      <c r="N5" s="12" t="n"/>
+      <c r="O5" s="12" t="n"/>
+      <c r="P5" s="13" t="n"/>
+      <c r="Q5" s="14">
+        <f>IF(C5="","",MAX(D5,IF(COUNT(E5:G5)=3,E5*F5*G5/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R5" s="14">
+        <f>IF(OR(Q5="",H5=""),"",Q5*H5)</f>
+        <v/>
+      </c>
+      <c r="S5" s="15">
+        <f>IF(R5="","",IF(R5&lt;=0,"",IF(ROUNDUP(R5,0)&gt;20,ROUNDUP(R5,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R5,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T5" s="15">
+        <f>IF(R5="","",IF(R5&lt;=0,"",IF(R5&gt;20,ROUNDUP(R5,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R5,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U5" s="16">
+        <f>IF(S5="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S5&lt;=T5,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V5" s="15">
+        <f>IF(U5="","",IF(U5="VPS",S5,T5))</f>
+        <v/>
+      </c>
+      <c r="W5" s="17">
+        <f>IF(C5="","",IF(I5&lt;&gt;"",I5*Q5,IF('THAM SỐ'!$C$4="US",IFERROR(V5/'THAM SỐ'!$C$13/H5,0),0)))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4">
@@ -1220,16 +1367,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C6="","",'DỮ LIỆU FASTMOSS'!C6)</f>
         <v/>
       </c>
-      <c r="C6" s="12" t="n"/>
-      <c r="D6" s="11" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="12" t="n"/>
       <c r="E6" s="12" t="n"/>
       <c r="F6" s="12" t="n"/>
       <c r="G6" s="12" t="n"/>
       <c r="H6" s="12" t="n"/>
-      <c r="I6" s="12" t="n"/>
-      <c r="J6" s="11" t="n"/>
-      <c r="K6" s="11" t="n"/>
-      <c r="L6" s="12" t="n"/>
+      <c r="I6" s="13" t="n"/>
+      <c r="J6" s="13" t="n"/>
+      <c r="K6" s="13" t="n"/>
+      <c r="L6" s="13" t="n"/>
+      <c r="M6" s="13" t="n"/>
+      <c r="N6" s="12" t="n"/>
+      <c r="O6" s="12" t="n"/>
+      <c r="P6" s="13" t="n"/>
+      <c r="Q6" s="14">
+        <f>IF(C6="","",MAX(D6,IF(COUNT(E6:G6)=3,E6*F6*G6/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R6" s="14">
+        <f>IF(OR(Q6="",H6=""),"",Q6*H6)</f>
+        <v/>
+      </c>
+      <c r="S6" s="15">
+        <f>IF(R6="","",IF(R6&lt;=0,"",IF(ROUNDUP(R6,0)&gt;20,ROUNDUP(R6,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R6,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T6" s="15">
+        <f>IF(R6="","",IF(R6&lt;=0,"",IF(R6&gt;20,ROUNDUP(R6,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R6,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U6" s="16">
+        <f>IF(S6="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S6&lt;=T6,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V6" s="15">
+        <f>IF(U6="","",IF(U6="VPS",S6,T6))</f>
+        <v/>
+      </c>
+      <c r="W6" s="17">
+        <f>IF(C6="","",IF(I6&lt;&gt;"",I6*Q6,IF('THAM SỐ'!$C$4="US",IFERROR(V6/'THAM SỐ'!$C$13/H6,0),0)))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4">
@@ -1240,16 +1419,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C7="","",'DỮ LIỆU FASTMOSS'!C7)</f>
         <v/>
       </c>
-      <c r="C7" s="12" t="n"/>
-      <c r="D7" s="11" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="12" t="n"/>
       <c r="E7" s="12" t="n"/>
       <c r="F7" s="12" t="n"/>
       <c r="G7" s="12" t="n"/>
       <c r="H7" s="12" t="n"/>
-      <c r="I7" s="12" t="n"/>
-      <c r="J7" s="11" t="n"/>
-      <c r="K7" s="11" t="n"/>
-      <c r="L7" s="12" t="n"/>
+      <c r="I7" s="13" t="n"/>
+      <c r="J7" s="13" t="n"/>
+      <c r="K7" s="13" t="n"/>
+      <c r="L7" s="13" t="n"/>
+      <c r="M7" s="13" t="n"/>
+      <c r="N7" s="12" t="n"/>
+      <c r="O7" s="12" t="n"/>
+      <c r="P7" s="13" t="n"/>
+      <c r="Q7" s="14">
+        <f>IF(C7="","",MAX(D7,IF(COUNT(E7:G7)=3,E7*F7*G7/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R7" s="14">
+        <f>IF(OR(Q7="",H7=""),"",Q7*H7)</f>
+        <v/>
+      </c>
+      <c r="S7" s="15">
+        <f>IF(R7="","",IF(R7&lt;=0,"",IF(ROUNDUP(R7,0)&gt;20,ROUNDUP(R7,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R7,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T7" s="15">
+        <f>IF(R7="","",IF(R7&lt;=0,"",IF(R7&gt;20,ROUNDUP(R7,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R7,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U7" s="16">
+        <f>IF(S7="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S7&lt;=T7,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V7" s="15">
+        <f>IF(U7="","",IF(U7="VPS",S7,T7))</f>
+        <v/>
+      </c>
+      <c r="W7" s="17">
+        <f>IF(C7="","",IF(I7&lt;&gt;"",I7*Q7,IF('THAM SỐ'!$C$4="US",IFERROR(V7/'THAM SỐ'!$C$13/H7,0),0)))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4">
@@ -1260,16 +1471,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C8="","",'DỮ LIỆU FASTMOSS'!C8)</f>
         <v/>
       </c>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="11" t="n"/>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="12" t="n"/>
       <c r="E8" s="12" t="n"/>
       <c r="F8" s="12" t="n"/>
       <c r="G8" s="12" t="n"/>
       <c r="H8" s="12" t="n"/>
-      <c r="I8" s="12" t="n"/>
-      <c r="J8" s="11" t="n"/>
-      <c r="K8" s="11" t="n"/>
-      <c r="L8" s="12" t="n"/>
+      <c r="I8" s="13" t="n"/>
+      <c r="J8" s="13" t="n"/>
+      <c r="K8" s="13" t="n"/>
+      <c r="L8" s="13" t="n"/>
+      <c r="M8" s="13" t="n"/>
+      <c r="N8" s="12" t="n"/>
+      <c r="O8" s="12" t="n"/>
+      <c r="P8" s="13" t="n"/>
+      <c r="Q8" s="14">
+        <f>IF(C8="","",MAX(D8,IF(COUNT(E8:G8)=3,E8*F8*G8/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R8" s="14">
+        <f>IF(OR(Q8="",H8=""),"",Q8*H8)</f>
+        <v/>
+      </c>
+      <c r="S8" s="15">
+        <f>IF(R8="","",IF(R8&lt;=0,"",IF(ROUNDUP(R8,0)&gt;20,ROUNDUP(R8,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R8,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T8" s="15">
+        <f>IF(R8="","",IF(R8&lt;=0,"",IF(R8&gt;20,ROUNDUP(R8,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R8,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U8" s="16">
+        <f>IF(S8="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S8&lt;=T8,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V8" s="15">
+        <f>IF(U8="","",IF(U8="VPS",S8,T8))</f>
+        <v/>
+      </c>
+      <c r="W8" s="17">
+        <f>IF(C8="","",IF(I8&lt;&gt;"",I8*Q8,IF('THAM SỐ'!$C$4="US",IFERROR(V8/'THAM SỐ'!$C$13/H8,0),0)))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4">
@@ -1280,16 +1523,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C9="","",'DỮ LIỆU FASTMOSS'!C9)</f>
         <v/>
       </c>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="11" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="12" t="n"/>
       <c r="E9" s="12" t="n"/>
       <c r="F9" s="12" t="n"/>
       <c r="G9" s="12" t="n"/>
       <c r="H9" s="12" t="n"/>
-      <c r="I9" s="12" t="n"/>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="11" t="n"/>
-      <c r="L9" s="12" t="n"/>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="13" t="n"/>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="13" t="n"/>
+      <c r="M9" s="13" t="n"/>
+      <c r="N9" s="12" t="n"/>
+      <c r="O9" s="12" t="n"/>
+      <c r="P9" s="13" t="n"/>
+      <c r="Q9" s="14">
+        <f>IF(C9="","",MAX(D9,IF(COUNT(E9:G9)=3,E9*F9*G9/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R9" s="14">
+        <f>IF(OR(Q9="",H9=""),"",Q9*H9)</f>
+        <v/>
+      </c>
+      <c r="S9" s="15">
+        <f>IF(R9="","",IF(R9&lt;=0,"",IF(ROUNDUP(R9,0)&gt;20,ROUNDUP(R9,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R9,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T9" s="15">
+        <f>IF(R9="","",IF(R9&lt;=0,"",IF(R9&gt;20,ROUNDUP(R9,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R9,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U9" s="16">
+        <f>IF(S9="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S9&lt;=T9,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V9" s="15">
+        <f>IF(U9="","",IF(U9="VPS",S9,T9))</f>
+        <v/>
+      </c>
+      <c r="W9" s="17">
+        <f>IF(C9="","",IF(I9&lt;&gt;"",I9*Q9,IF('THAM SỐ'!$C$4="US",IFERROR(V9/'THAM SỐ'!$C$13/H9,0),0)))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4">
@@ -1300,16 +1575,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C10="","",'DỮ LIỆU FASTMOSS'!C10)</f>
         <v/>
       </c>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="11" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="12" t="n"/>
       <c r="E10" s="12" t="n"/>
       <c r="F10" s="12" t="n"/>
       <c r="G10" s="12" t="n"/>
       <c r="H10" s="12" t="n"/>
-      <c r="I10" s="12" t="n"/>
-      <c r="J10" s="11" t="n"/>
-      <c r="K10" s="11" t="n"/>
-      <c r="L10" s="12" t="n"/>
+      <c r="I10" s="13" t="n"/>
+      <c r="J10" s="13" t="n"/>
+      <c r="K10" s="13" t="n"/>
+      <c r="L10" s="13" t="n"/>
+      <c r="M10" s="13" t="n"/>
+      <c r="N10" s="12" t="n"/>
+      <c r="O10" s="12" t="n"/>
+      <c r="P10" s="13" t="n"/>
+      <c r="Q10" s="14">
+        <f>IF(C10="","",MAX(D10,IF(COUNT(E10:G10)=3,E10*F10*G10/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R10" s="14">
+        <f>IF(OR(Q10="",H10=""),"",Q10*H10)</f>
+        <v/>
+      </c>
+      <c r="S10" s="15">
+        <f>IF(R10="","",IF(R10&lt;=0,"",IF(ROUNDUP(R10,0)&gt;20,ROUNDUP(R10,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R10,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T10" s="15">
+        <f>IF(R10="","",IF(R10&lt;=0,"",IF(R10&gt;20,ROUNDUP(R10,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R10,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U10" s="16">
+        <f>IF(S10="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S10&lt;=T10,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V10" s="15">
+        <f>IF(U10="","",IF(U10="VPS",S10,T10))</f>
+        <v/>
+      </c>
+      <c r="W10" s="17">
+        <f>IF(C10="","",IF(I10&lt;&gt;"",I10*Q10,IF('THAM SỐ'!$C$4="US",IFERROR(V10/'THAM SỐ'!$C$13/H10,0),0)))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4">
@@ -1320,16 +1627,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C11="","",'DỮ LIỆU FASTMOSS'!C11)</f>
         <v/>
       </c>
-      <c r="C11" s="12" t="n"/>
-      <c r="D11" s="11" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="12" t="n"/>
       <c r="E11" s="12" t="n"/>
       <c r="F11" s="12" t="n"/>
       <c r="G11" s="12" t="n"/>
       <c r="H11" s="12" t="n"/>
-      <c r="I11" s="12" t="n"/>
-      <c r="J11" s="11" t="n"/>
-      <c r="K11" s="11" t="n"/>
-      <c r="L11" s="12" t="n"/>
+      <c r="I11" s="13" t="n"/>
+      <c r="J11" s="13" t="n"/>
+      <c r="K11" s="13" t="n"/>
+      <c r="L11" s="13" t="n"/>
+      <c r="M11" s="13" t="n"/>
+      <c r="N11" s="12" t="n"/>
+      <c r="O11" s="12" t="n"/>
+      <c r="P11" s="13" t="n"/>
+      <c r="Q11" s="14">
+        <f>IF(C11="","",MAX(D11,IF(COUNT(E11:G11)=3,E11*F11*G11/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R11" s="14">
+        <f>IF(OR(Q11="",H11=""),"",Q11*H11)</f>
+        <v/>
+      </c>
+      <c r="S11" s="15">
+        <f>IF(R11="","",IF(R11&lt;=0,"",IF(ROUNDUP(R11,0)&gt;20,ROUNDUP(R11,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R11,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T11" s="15">
+        <f>IF(R11="","",IF(R11&lt;=0,"",IF(R11&gt;20,ROUNDUP(R11,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R11,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U11" s="16">
+        <f>IF(S11="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S11&lt;=T11,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V11" s="15">
+        <f>IF(U11="","",IF(U11="VPS",S11,T11))</f>
+        <v/>
+      </c>
+      <c r="W11" s="17">
+        <f>IF(C11="","",IF(I11&lt;&gt;"",I11*Q11,IF('THAM SỐ'!$C$4="US",IFERROR(V11/'THAM SỐ'!$C$13/H11,0),0)))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4">
@@ -1340,16 +1679,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C12="","",'DỮ LIỆU FASTMOSS'!C12)</f>
         <v/>
       </c>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="11" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="12" t="n"/>
       <c r="E12" s="12" t="n"/>
       <c r="F12" s="12" t="n"/>
       <c r="G12" s="12" t="n"/>
       <c r="H12" s="12" t="n"/>
-      <c r="I12" s="12" t="n"/>
-      <c r="J12" s="11" t="n"/>
-      <c r="K12" s="11" t="n"/>
-      <c r="L12" s="12" t="n"/>
+      <c r="I12" s="13" t="n"/>
+      <c r="J12" s="13" t="n"/>
+      <c r="K12" s="13" t="n"/>
+      <c r="L12" s="13" t="n"/>
+      <c r="M12" s="13" t="n"/>
+      <c r="N12" s="12" t="n"/>
+      <c r="O12" s="12" t="n"/>
+      <c r="P12" s="13" t="n"/>
+      <c r="Q12" s="14">
+        <f>IF(C12="","",MAX(D12,IF(COUNT(E12:G12)=3,E12*F12*G12/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R12" s="14">
+        <f>IF(OR(Q12="",H12=""),"",Q12*H12)</f>
+        <v/>
+      </c>
+      <c r="S12" s="15">
+        <f>IF(R12="","",IF(R12&lt;=0,"",IF(ROUNDUP(R12,0)&gt;20,ROUNDUP(R12,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R12,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T12" s="15">
+        <f>IF(R12="","",IF(R12&lt;=0,"",IF(R12&gt;20,ROUNDUP(R12,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R12,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U12" s="16">
+        <f>IF(S12="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S12&lt;=T12,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V12" s="15">
+        <f>IF(U12="","",IF(U12="VPS",S12,T12))</f>
+        <v/>
+      </c>
+      <c r="W12" s="17">
+        <f>IF(C12="","",IF(I12&lt;&gt;"",I12*Q12,IF('THAM SỐ'!$C$4="US",IFERROR(V12/'THAM SỐ'!$C$13/H12,0),0)))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4">
@@ -1360,16 +1731,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C13="","",'DỮ LIỆU FASTMOSS'!C13)</f>
         <v/>
       </c>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="11" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="12" t="n"/>
       <c r="E13" s="12" t="n"/>
       <c r="F13" s="12" t="n"/>
       <c r="G13" s="12" t="n"/>
       <c r="H13" s="12" t="n"/>
-      <c r="I13" s="12" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n"/>
-      <c r="L13" s="12" t="n"/>
+      <c r="I13" s="13" t="n"/>
+      <c r="J13" s="13" t="n"/>
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="13" t="n"/>
+      <c r="M13" s="13" t="n"/>
+      <c r="N13" s="12" t="n"/>
+      <c r="O13" s="12" t="n"/>
+      <c r="P13" s="13" t="n"/>
+      <c r="Q13" s="14">
+        <f>IF(C13="","",MAX(D13,IF(COUNT(E13:G13)=3,E13*F13*G13/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R13" s="14">
+        <f>IF(OR(Q13="",H13=""),"",Q13*H13)</f>
+        <v/>
+      </c>
+      <c r="S13" s="15">
+        <f>IF(R13="","",IF(R13&lt;=0,"",IF(ROUNDUP(R13,0)&gt;20,ROUNDUP(R13,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R13,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T13" s="15">
+        <f>IF(R13="","",IF(R13&lt;=0,"",IF(R13&gt;20,ROUNDUP(R13,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R13,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U13" s="16">
+        <f>IF(S13="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S13&lt;=T13,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V13" s="15">
+        <f>IF(U13="","",IF(U13="VPS",S13,T13))</f>
+        <v/>
+      </c>
+      <c r="W13" s="17">
+        <f>IF(C13="","",IF(I13&lt;&gt;"",I13*Q13,IF('THAM SỐ'!$C$4="US",IFERROR(V13/'THAM SỐ'!$C$13/H13,0),0)))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4">
@@ -1380,16 +1783,48 @@
         <f>IF('DỮ LIỆU FASTMOSS'!C14="","",'DỮ LIỆU FASTMOSS'!C14)</f>
         <v/>
       </c>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="11" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="12" t="n"/>
       <c r="E14" s="12" t="n"/>
       <c r="F14" s="12" t="n"/>
       <c r="G14" s="12" t="n"/>
       <c r="H14" s="12" t="n"/>
-      <c r="I14" s="12" t="n"/>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="11" t="n"/>
-      <c r="L14" s="12" t="n"/>
+      <c r="I14" s="13" t="n"/>
+      <c r="J14" s="13" t="n"/>
+      <c r="K14" s="13" t="n"/>
+      <c r="L14" s="13" t="n"/>
+      <c r="M14" s="13" t="n"/>
+      <c r="N14" s="12" t="n"/>
+      <c r="O14" s="12" t="n"/>
+      <c r="P14" s="13" t="n"/>
+      <c r="Q14" s="14">
+        <f>IF(C14="","",MAX(D14,IF(COUNT(E14:G14)=3,E14*F14*G14/5000,0)))</f>
+        <v/>
+      </c>
+      <c r="R14" s="14">
+        <f>IF(OR(Q14="",H14=""),"",Q14*H14)</f>
+        <v/>
+      </c>
+      <c r="S14" s="15">
+        <f>IF(R14="","",IF(R14&lt;=0,"",IF(ROUNDUP(R14,0)&gt;20,ROUNDUP(R14,0)*'CƯỚC VẬN CHUYỂN'!$C$27,INDEX('CƯỚC VẬN CHUYỂN'!$C$5:$C$24,MATCH(MAX(1,ROUNDUP(R14,0)),'CƯỚC VẬN CHUYỂN'!$B$5:$B$24,0)))))</f>
+        <v/>
+      </c>
+      <c r="T14" s="15">
+        <f>IF(R14="","",IF(R14&lt;=0,"",IF(R14&gt;20,ROUNDUP(R14,0)*'CƯỚC VẬN CHUYỂN'!$G$37,INDEX('CƯỚC VẬN CHUYỂN'!$G$5:$G$36,MATCH(MAX(0.5,CEILING(R14,0.5)),'CƯỚC VẬN CHUYỂN'!$F$5:$F$36,0)))))</f>
+        <v/>
+      </c>
+      <c r="U14" s="16">
+        <f>IF(S14="","",IF('THAM SỐ'!$C$14="VPS","VPS",IF('THAM SỐ'!$C$14="AM","AM",IF(S14&lt;=T14,"VPS","AM"))))</f>
+        <v/>
+      </c>
+      <c r="V14" s="15">
+        <f>IF(U14="","",IF(U14="VPS",S14,T14))</f>
+        <v/>
+      </c>
+      <c r="W14" s="17">
+        <f>IF(C14="","",IF(I14&lt;&gt;"",I14*Q14,IF('THAM SỐ'!$C$4="US",IFERROR(V14/'THAM SỐ'!$C$13/H14,0),0)))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1438,87 +1873,87 @@
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Mã SP</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Tên sản phẩm</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Loại</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Giá bán dùng để tính</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Giá vốn hàng về tới khách</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Phí sàn (giao dịch, hoa hồng, xử lý, thuế)</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>Hoa hồng affiliate</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>Vận hành và marketing mỗi đơn</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="10" t="inlineStr">
         <is>
           <t>Hoàn, hủy, hỏng</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="10" t="inlineStr">
         <is>
           <t>Lợi nhuận đơn tự nhiên</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>Biên đơn tự nhiên</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="L4" s="10" t="inlineStr">
         <is>
           <t>Lợi nhuận đơn affiliate</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="M4" s="10" t="inlineStr">
         <is>
           <t>Lợi nhuận đơn quảng cáo</t>
         </is>
       </c>
-      <c r="N4" s="9" t="inlineStr">
+      <c r="N4" s="10" t="inlineStr">
         <is>
           <t>Giá nhập tối đa để đạt biên</t>
         </is>
       </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="O4" s="10" t="inlineStr">
         <is>
           <t>Giá bán đề xuất để đạt biên</t>
         </is>
       </c>
-      <c r="P4" s="9" t="inlineStr">
+      <c r="P4" s="10" t="inlineStr">
         <is>
           <t>Vị trí giá đề xuất so với thị trường</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
+      <c r="Q4" s="10" t="inlineStr">
         <is>
           <t>Kết luận</t>
         </is>
@@ -1537,51 +1972,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B5="","",'DỮ LIỆU FASTMOSS'!B5)</f>
         <v/>
       </c>
-      <c r="D5" s="13">
-        <f>IF(A5="","",IF('NHẬP HÀNG'!L5&lt;&gt;"",'NHẬP HÀNG'!L5,'DỮ LIỆU FASTMOSS'!E5))</f>
-        <v/>
-      </c>
-      <c r="E5" s="13">
-        <f>IF(OR(A5="",'NHẬP HÀNG'!C5=""),"",'NHẬP HÀNG'!C5+'NHẬP HÀNG'!D5*'NHẬP HÀNG'!E5+'NHẬP HÀNG'!F5+'NHẬP HÀNG'!G5+'NHẬP HÀNG'!H5+'NHẬP HÀNG'!I5)</f>
-        <v/>
-      </c>
-      <c r="F5" s="13">
+      <c r="D5" s="18">
+        <f>IF(A5="","",IF('NHẬP HÀNG'!P5&lt;&gt;"",'NHẬP HÀNG'!P5,'DỮ LIỆU FASTMOSS'!E5))</f>
+        <v/>
+      </c>
+      <c r="E5" s="18">
+        <f>IF(OR(A5="",'NHẬP HÀNG'!C5=""),"",'NHẬP HÀNG'!C5+'NHẬP HÀNG'!W5+'NHẬP HÀNG'!J5+'NHẬP HÀNG'!K5+'NHẬP HÀNG'!L5+'NHẬP HÀNG'!M5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="18">
         <f>IF(OR(A5="",D5=""),"",D5*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="18">
         <f>IF(OR(A5="",D5=""),"",D5*'DỮ LIỆU FASTMOSS'!I5/100)</f>
         <v/>
       </c>
-      <c r="H5" s="13">
+      <c r="H5" s="18">
         <f>IF(A5="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I5" s="13">
+      <c r="I5" s="18">
         <f>IF(OR(A5="",D5=""),"",D5*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J5" s="14">
+      <c r="J5" s="19">
         <f>IF(OR(E5="",D5=""),"",D5-E5-F5-H5-I5)</f>
         <v/>
       </c>
-      <c r="K5" s="15">
+      <c r="K5" s="20">
         <f>IF(J5="","",IFERROR(J5/D5,""))</f>
         <v/>
       </c>
-      <c r="L5" s="13">
+      <c r="L5" s="18">
         <f>IF(J5="","",J5-G5)</f>
         <v/>
       </c>
-      <c r="M5" s="13">
+      <c r="M5" s="18">
         <f>IF(J5="","",J5-D5*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N5" s="14">
+      <c r="N5" s="19">
         <f>IF(OR(E5="",D5=""),"",D5*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H5+(E5-'NHẬP HÀNG'!C5)))</f>
         <v/>
       </c>
-      <c r="O5" s="14">
+      <c r="O5" s="19">
         <f>IF(E5="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E5+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H5)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -1589,7 +2024,7 @@
         <f>IF(OR(NOT(ISNUMBER(O5)),'DỮ LIỆU FASTMOSS'!D5=""),"",IF(O5&lt;'DỮ LIỆU FASTMOSS'!D5,"Thấp hơn mọi đối thủ",IF(O5&lt;='DỮ LIỆU FASTMOSS'!E5,"Dưới hoặc bằng trung vị",IF(O5&lt;='DỮ LIỆU FASTMOSS'!F5,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q5" s="16">
+      <c r="Q5" s="21">
         <f>IF(A5="","",IF(E5="","Chờ nhập hàng",IF(AND(K5&gt;='THAM SỐ'!C6,NOT(P5="Cao hơn mọi đối thủ")),"Làm",IF(J5&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -1607,51 +2042,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B6="","",'DỮ LIỆU FASTMOSS'!B6)</f>
         <v/>
       </c>
-      <c r="D6" s="13">
-        <f>IF(A6="","",IF('NHẬP HÀNG'!L6&lt;&gt;"",'NHẬP HÀNG'!L6,'DỮ LIỆU FASTMOSS'!E6))</f>
-        <v/>
-      </c>
-      <c r="E6" s="13">
-        <f>IF(OR(A6="",'NHẬP HÀNG'!C6=""),"",'NHẬP HÀNG'!C6+'NHẬP HÀNG'!D6*'NHẬP HÀNG'!E6+'NHẬP HÀNG'!F6+'NHẬP HÀNG'!G6+'NHẬP HÀNG'!H6+'NHẬP HÀNG'!I6)</f>
-        <v/>
-      </c>
-      <c r="F6" s="13">
+      <c r="D6" s="18">
+        <f>IF(A6="","",IF('NHẬP HÀNG'!P6&lt;&gt;"",'NHẬP HÀNG'!P6,'DỮ LIỆU FASTMOSS'!E6))</f>
+        <v/>
+      </c>
+      <c r="E6" s="18">
+        <f>IF(OR(A6="",'NHẬP HÀNG'!C6=""),"",'NHẬP HÀNG'!C6+'NHẬP HÀNG'!W6+'NHẬP HÀNG'!J6+'NHẬP HÀNG'!K6+'NHẬP HÀNG'!L6+'NHẬP HÀNG'!M6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="18">
         <f>IF(OR(A6="",D6=""),"",D6*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="18">
         <f>IF(OR(A6="",D6=""),"",D6*'DỮ LIỆU FASTMOSS'!I6/100)</f>
         <v/>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="18">
         <f>IF(A6="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I6" s="13">
+      <c r="I6" s="18">
         <f>IF(OR(A6="",D6=""),"",D6*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J6" s="14">
+      <c r="J6" s="19">
         <f>IF(OR(E6="",D6=""),"",D6-E6-F6-H6-I6)</f>
         <v/>
       </c>
-      <c r="K6" s="15">
+      <c r="K6" s="20">
         <f>IF(J6="","",IFERROR(J6/D6,""))</f>
         <v/>
       </c>
-      <c r="L6" s="13">
+      <c r="L6" s="18">
         <f>IF(J6="","",J6-G6)</f>
         <v/>
       </c>
-      <c r="M6" s="13">
+      <c r="M6" s="18">
         <f>IF(J6="","",J6-D6*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N6" s="14">
+      <c r="N6" s="19">
         <f>IF(OR(E6="",D6=""),"",D6*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H6+(E6-'NHẬP HÀNG'!C6)))</f>
         <v/>
       </c>
-      <c r="O6" s="14">
+      <c r="O6" s="19">
         <f>IF(E6="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E6+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H6)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -1659,7 +2094,7 @@
         <f>IF(OR(NOT(ISNUMBER(O6)),'DỮ LIỆU FASTMOSS'!D6=""),"",IF(O6&lt;'DỮ LIỆU FASTMOSS'!D6,"Thấp hơn mọi đối thủ",IF(O6&lt;='DỮ LIỆU FASTMOSS'!E6,"Dưới hoặc bằng trung vị",IF(O6&lt;='DỮ LIỆU FASTMOSS'!F6,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q6" s="16">
+      <c r="Q6" s="21">
         <f>IF(A6="","",IF(E6="","Chờ nhập hàng",IF(AND(K6&gt;='THAM SỐ'!C6,NOT(P6="Cao hơn mọi đối thủ")),"Làm",IF(J6&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -1677,51 +2112,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B7="","",'DỮ LIỆU FASTMOSS'!B7)</f>
         <v/>
       </c>
-      <c r="D7" s="13">
-        <f>IF(A7="","",IF('NHẬP HÀNG'!L7&lt;&gt;"",'NHẬP HÀNG'!L7,'DỮ LIỆU FASTMOSS'!E7))</f>
-        <v/>
-      </c>
-      <c r="E7" s="13">
-        <f>IF(OR(A7="",'NHẬP HÀNG'!C7=""),"",'NHẬP HÀNG'!C7+'NHẬP HÀNG'!D7*'NHẬP HÀNG'!E7+'NHẬP HÀNG'!F7+'NHẬP HÀNG'!G7+'NHẬP HÀNG'!H7+'NHẬP HÀNG'!I7)</f>
-        <v/>
-      </c>
-      <c r="F7" s="13">
+      <c r="D7" s="18">
+        <f>IF(A7="","",IF('NHẬP HÀNG'!P7&lt;&gt;"",'NHẬP HÀNG'!P7,'DỮ LIỆU FASTMOSS'!E7))</f>
+        <v/>
+      </c>
+      <c r="E7" s="18">
+        <f>IF(OR(A7="",'NHẬP HÀNG'!C7=""),"",'NHẬP HÀNG'!C7+'NHẬP HÀNG'!W7+'NHẬP HÀNG'!J7+'NHẬP HÀNG'!K7+'NHẬP HÀNG'!L7+'NHẬP HÀNG'!M7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="18">
         <f>IF(OR(A7="",D7=""),"",D7*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="18">
         <f>IF(OR(A7="",D7=""),"",D7*'DỮ LIỆU FASTMOSS'!I7/100)</f>
         <v/>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="18">
         <f>IF(A7="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I7" s="13">
+      <c r="I7" s="18">
         <f>IF(OR(A7="",D7=""),"",D7*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J7" s="14">
+      <c r="J7" s="19">
         <f>IF(OR(E7="",D7=""),"",D7-E7-F7-H7-I7)</f>
         <v/>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="20">
         <f>IF(J7="","",IFERROR(J7/D7,""))</f>
         <v/>
       </c>
-      <c r="L7" s="13">
+      <c r="L7" s="18">
         <f>IF(J7="","",J7-G7)</f>
         <v/>
       </c>
-      <c r="M7" s="13">
+      <c r="M7" s="18">
         <f>IF(J7="","",J7-D7*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N7" s="14">
+      <c r="N7" s="19">
         <f>IF(OR(E7="",D7=""),"",D7*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H7+(E7-'NHẬP HÀNG'!C7)))</f>
         <v/>
       </c>
-      <c r="O7" s="14">
+      <c r="O7" s="19">
         <f>IF(E7="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E7+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H7)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -1729,7 +2164,7 @@
         <f>IF(OR(NOT(ISNUMBER(O7)),'DỮ LIỆU FASTMOSS'!D7=""),"",IF(O7&lt;'DỮ LIỆU FASTMOSS'!D7,"Thấp hơn mọi đối thủ",IF(O7&lt;='DỮ LIỆU FASTMOSS'!E7,"Dưới hoặc bằng trung vị",IF(O7&lt;='DỮ LIỆU FASTMOSS'!F7,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q7" s="16">
+      <c r="Q7" s="21">
         <f>IF(A7="","",IF(E7="","Chờ nhập hàng",IF(AND(K7&gt;='THAM SỐ'!C6,NOT(P7="Cao hơn mọi đối thủ")),"Làm",IF(J7&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -1747,51 +2182,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B8="","",'DỮ LIỆU FASTMOSS'!B8)</f>
         <v/>
       </c>
-      <c r="D8" s="13">
-        <f>IF(A8="","",IF('NHẬP HÀNG'!L8&lt;&gt;"",'NHẬP HÀNG'!L8,'DỮ LIỆU FASTMOSS'!E8))</f>
-        <v/>
-      </c>
-      <c r="E8" s="13">
-        <f>IF(OR(A8="",'NHẬP HÀNG'!C8=""),"",'NHẬP HÀNG'!C8+'NHẬP HÀNG'!D8*'NHẬP HÀNG'!E8+'NHẬP HÀNG'!F8+'NHẬP HÀNG'!G8+'NHẬP HÀNG'!H8+'NHẬP HÀNG'!I8)</f>
-        <v/>
-      </c>
-      <c r="F8" s="13">
+      <c r="D8" s="18">
+        <f>IF(A8="","",IF('NHẬP HÀNG'!P8&lt;&gt;"",'NHẬP HÀNG'!P8,'DỮ LIỆU FASTMOSS'!E8))</f>
+        <v/>
+      </c>
+      <c r="E8" s="18">
+        <f>IF(OR(A8="",'NHẬP HÀNG'!C8=""),"",'NHẬP HÀNG'!C8+'NHẬP HÀNG'!W8+'NHẬP HÀNG'!J8+'NHẬP HÀNG'!K8+'NHẬP HÀNG'!L8+'NHẬP HÀNG'!M8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="18">
         <f>IF(OR(A8="",D8=""),"",D8*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="18">
         <f>IF(OR(A8="",D8=""),"",D8*'DỮ LIỆU FASTMOSS'!I8/100)</f>
         <v/>
       </c>
-      <c r="H8" s="13">
+      <c r="H8" s="18">
         <f>IF(A8="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I8" s="13">
+      <c r="I8" s="18">
         <f>IF(OR(A8="",D8=""),"",D8*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J8" s="14">
+      <c r="J8" s="19">
         <f>IF(OR(E8="",D8=""),"",D8-E8-F8-H8-I8)</f>
         <v/>
       </c>
-      <c r="K8" s="15">
+      <c r="K8" s="20">
         <f>IF(J8="","",IFERROR(J8/D8,""))</f>
         <v/>
       </c>
-      <c r="L8" s="13">
+      <c r="L8" s="18">
         <f>IF(J8="","",J8-G8)</f>
         <v/>
       </c>
-      <c r="M8" s="13">
+      <c r="M8" s="18">
         <f>IF(J8="","",J8-D8*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N8" s="14">
+      <c r="N8" s="19">
         <f>IF(OR(E8="",D8=""),"",D8*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H8+(E8-'NHẬP HÀNG'!C8)))</f>
         <v/>
       </c>
-      <c r="O8" s="14">
+      <c r="O8" s="19">
         <f>IF(E8="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E8+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H8)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -1799,7 +2234,7 @@
         <f>IF(OR(NOT(ISNUMBER(O8)),'DỮ LIỆU FASTMOSS'!D8=""),"",IF(O8&lt;'DỮ LIỆU FASTMOSS'!D8,"Thấp hơn mọi đối thủ",IF(O8&lt;='DỮ LIỆU FASTMOSS'!E8,"Dưới hoặc bằng trung vị",IF(O8&lt;='DỮ LIỆU FASTMOSS'!F8,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q8" s="16">
+      <c r="Q8" s="21">
         <f>IF(A8="","",IF(E8="","Chờ nhập hàng",IF(AND(K8&gt;='THAM SỐ'!C6,NOT(P8="Cao hơn mọi đối thủ")),"Làm",IF(J8&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -1817,51 +2252,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B9="","",'DỮ LIỆU FASTMOSS'!B9)</f>
         <v/>
       </c>
-      <c r="D9" s="13">
-        <f>IF(A9="","",IF('NHẬP HÀNG'!L9&lt;&gt;"",'NHẬP HÀNG'!L9,'DỮ LIỆU FASTMOSS'!E9))</f>
-        <v/>
-      </c>
-      <c r="E9" s="13">
-        <f>IF(OR(A9="",'NHẬP HÀNG'!C9=""),"",'NHẬP HÀNG'!C9+'NHẬP HÀNG'!D9*'NHẬP HÀNG'!E9+'NHẬP HÀNG'!F9+'NHẬP HÀNG'!G9+'NHẬP HÀNG'!H9+'NHẬP HÀNG'!I9)</f>
-        <v/>
-      </c>
-      <c r="F9" s="13">
+      <c r="D9" s="18">
+        <f>IF(A9="","",IF('NHẬP HÀNG'!P9&lt;&gt;"",'NHẬP HÀNG'!P9,'DỮ LIỆU FASTMOSS'!E9))</f>
+        <v/>
+      </c>
+      <c r="E9" s="18">
+        <f>IF(OR(A9="",'NHẬP HÀNG'!C9=""),"",'NHẬP HÀNG'!C9+'NHẬP HÀNG'!W9+'NHẬP HÀNG'!J9+'NHẬP HÀNG'!K9+'NHẬP HÀNG'!L9+'NHẬP HÀNG'!M9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="18">
         <f>IF(OR(A9="",D9=""),"",D9*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="18">
         <f>IF(OR(A9="",D9=""),"",D9*'DỮ LIỆU FASTMOSS'!I9/100)</f>
         <v/>
       </c>
-      <c r="H9" s="13">
+      <c r="H9" s="18">
         <f>IF(A9="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I9" s="13">
+      <c r="I9" s="18">
         <f>IF(OR(A9="",D9=""),"",D9*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="19">
         <f>IF(OR(E9="",D9=""),"",D9-E9-F9-H9-I9)</f>
         <v/>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="20">
         <f>IF(J9="","",IFERROR(J9/D9,""))</f>
         <v/>
       </c>
-      <c r="L9" s="13">
+      <c r="L9" s="18">
         <f>IF(J9="","",J9-G9)</f>
         <v/>
       </c>
-      <c r="M9" s="13">
+      <c r="M9" s="18">
         <f>IF(J9="","",J9-D9*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N9" s="14">
+      <c r="N9" s="19">
         <f>IF(OR(E9="",D9=""),"",D9*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H9+(E9-'NHẬP HÀNG'!C9)))</f>
         <v/>
       </c>
-      <c r="O9" s="14">
+      <c r="O9" s="19">
         <f>IF(E9="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E9+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H9)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -1869,7 +2304,7 @@
         <f>IF(OR(NOT(ISNUMBER(O9)),'DỮ LIỆU FASTMOSS'!D9=""),"",IF(O9&lt;'DỮ LIỆU FASTMOSS'!D9,"Thấp hơn mọi đối thủ",IF(O9&lt;='DỮ LIỆU FASTMOSS'!E9,"Dưới hoặc bằng trung vị",IF(O9&lt;='DỮ LIỆU FASTMOSS'!F9,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q9" s="16">
+      <c r="Q9" s="21">
         <f>IF(A9="","",IF(E9="","Chờ nhập hàng",IF(AND(K9&gt;='THAM SỐ'!C6,NOT(P9="Cao hơn mọi đối thủ")),"Làm",IF(J9&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -1887,51 +2322,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B10="","",'DỮ LIỆU FASTMOSS'!B10)</f>
         <v/>
       </c>
-      <c r="D10" s="13">
-        <f>IF(A10="","",IF('NHẬP HÀNG'!L10&lt;&gt;"",'NHẬP HÀNG'!L10,'DỮ LIỆU FASTMOSS'!E10))</f>
-        <v/>
-      </c>
-      <c r="E10" s="13">
-        <f>IF(OR(A10="",'NHẬP HÀNG'!C10=""),"",'NHẬP HÀNG'!C10+'NHẬP HÀNG'!D10*'NHẬP HÀNG'!E10+'NHẬP HÀNG'!F10+'NHẬP HÀNG'!G10+'NHẬP HÀNG'!H10+'NHẬP HÀNG'!I10)</f>
-        <v/>
-      </c>
-      <c r="F10" s="13">
+      <c r="D10" s="18">
+        <f>IF(A10="","",IF('NHẬP HÀNG'!P10&lt;&gt;"",'NHẬP HÀNG'!P10,'DỮ LIỆU FASTMOSS'!E10))</f>
+        <v/>
+      </c>
+      <c r="E10" s="18">
+        <f>IF(OR(A10="",'NHẬP HÀNG'!C10=""),"",'NHẬP HÀNG'!C10+'NHẬP HÀNG'!W10+'NHẬP HÀNG'!J10+'NHẬP HÀNG'!K10+'NHẬP HÀNG'!L10+'NHẬP HÀNG'!M10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="18">
         <f>IF(OR(A10="",D10=""),"",D10*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="18">
         <f>IF(OR(A10="",D10=""),"",D10*'DỮ LIỆU FASTMOSS'!I10/100)</f>
         <v/>
       </c>
-      <c r="H10" s="13">
+      <c r="H10" s="18">
         <f>IF(A10="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I10" s="13">
+      <c r="I10" s="18">
         <f>IF(OR(A10="",D10=""),"",D10*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J10" s="14">
+      <c r="J10" s="19">
         <f>IF(OR(E10="",D10=""),"",D10-E10-F10-H10-I10)</f>
         <v/>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="20">
         <f>IF(J10="","",IFERROR(J10/D10,""))</f>
         <v/>
       </c>
-      <c r="L10" s="13">
+      <c r="L10" s="18">
         <f>IF(J10="","",J10-G10)</f>
         <v/>
       </c>
-      <c r="M10" s="13">
+      <c r="M10" s="18">
         <f>IF(J10="","",J10-D10*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N10" s="14">
+      <c r="N10" s="19">
         <f>IF(OR(E10="",D10=""),"",D10*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H10+(E10-'NHẬP HÀNG'!C10)))</f>
         <v/>
       </c>
-      <c r="O10" s="14">
+      <c r="O10" s="19">
         <f>IF(E10="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E10+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H10)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -1939,7 +2374,7 @@
         <f>IF(OR(NOT(ISNUMBER(O10)),'DỮ LIỆU FASTMOSS'!D10=""),"",IF(O10&lt;'DỮ LIỆU FASTMOSS'!D10,"Thấp hơn mọi đối thủ",IF(O10&lt;='DỮ LIỆU FASTMOSS'!E10,"Dưới hoặc bằng trung vị",IF(O10&lt;='DỮ LIỆU FASTMOSS'!F10,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q10" s="16">
+      <c r="Q10" s="21">
         <f>IF(A10="","",IF(E10="","Chờ nhập hàng",IF(AND(K10&gt;='THAM SỐ'!C6,NOT(P10="Cao hơn mọi đối thủ")),"Làm",IF(J10&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -1957,51 +2392,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B11="","",'DỮ LIỆU FASTMOSS'!B11)</f>
         <v/>
       </c>
-      <c r="D11" s="13">
-        <f>IF(A11="","",IF('NHẬP HÀNG'!L11&lt;&gt;"",'NHẬP HÀNG'!L11,'DỮ LIỆU FASTMOSS'!E11))</f>
-        <v/>
-      </c>
-      <c r="E11" s="13">
-        <f>IF(OR(A11="",'NHẬP HÀNG'!C11=""),"",'NHẬP HÀNG'!C11+'NHẬP HÀNG'!D11*'NHẬP HÀNG'!E11+'NHẬP HÀNG'!F11+'NHẬP HÀNG'!G11+'NHẬP HÀNG'!H11+'NHẬP HÀNG'!I11)</f>
-        <v/>
-      </c>
-      <c r="F11" s="13">
+      <c r="D11" s="18">
+        <f>IF(A11="","",IF('NHẬP HÀNG'!P11&lt;&gt;"",'NHẬP HÀNG'!P11,'DỮ LIỆU FASTMOSS'!E11))</f>
+        <v/>
+      </c>
+      <c r="E11" s="18">
+        <f>IF(OR(A11="",'NHẬP HÀNG'!C11=""),"",'NHẬP HÀNG'!C11+'NHẬP HÀNG'!W11+'NHẬP HÀNG'!J11+'NHẬP HÀNG'!K11+'NHẬP HÀNG'!L11+'NHẬP HÀNG'!M11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="18">
         <f>IF(OR(A11="",D11=""),"",D11*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="18">
         <f>IF(OR(A11="",D11=""),"",D11*'DỮ LIỆU FASTMOSS'!I11/100)</f>
         <v/>
       </c>
-      <c r="H11" s="13">
+      <c r="H11" s="18">
         <f>IF(A11="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I11" s="13">
+      <c r="I11" s="18">
         <f>IF(OR(A11="",D11=""),"",D11*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J11" s="14">
+      <c r="J11" s="19">
         <f>IF(OR(E11="",D11=""),"",D11-E11-F11-H11-I11)</f>
         <v/>
       </c>
-      <c r="K11" s="15">
+      <c r="K11" s="20">
         <f>IF(J11="","",IFERROR(J11/D11,""))</f>
         <v/>
       </c>
-      <c r="L11" s="13">
+      <c r="L11" s="18">
         <f>IF(J11="","",J11-G11)</f>
         <v/>
       </c>
-      <c r="M11" s="13">
+      <c r="M11" s="18">
         <f>IF(J11="","",J11-D11*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N11" s="14">
+      <c r="N11" s="19">
         <f>IF(OR(E11="",D11=""),"",D11*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H11+(E11-'NHẬP HÀNG'!C11)))</f>
         <v/>
       </c>
-      <c r="O11" s="14">
+      <c r="O11" s="19">
         <f>IF(E11="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E11+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H11)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -2009,7 +2444,7 @@
         <f>IF(OR(NOT(ISNUMBER(O11)),'DỮ LIỆU FASTMOSS'!D11=""),"",IF(O11&lt;'DỮ LIỆU FASTMOSS'!D11,"Thấp hơn mọi đối thủ",IF(O11&lt;='DỮ LIỆU FASTMOSS'!E11,"Dưới hoặc bằng trung vị",IF(O11&lt;='DỮ LIỆU FASTMOSS'!F11,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q11" s="16">
+      <c r="Q11" s="21">
         <f>IF(A11="","",IF(E11="","Chờ nhập hàng",IF(AND(K11&gt;='THAM SỐ'!C6,NOT(P11="Cao hơn mọi đối thủ")),"Làm",IF(J11&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -2027,51 +2462,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B12="","",'DỮ LIỆU FASTMOSS'!B12)</f>
         <v/>
       </c>
-      <c r="D12" s="13">
-        <f>IF(A12="","",IF('NHẬP HÀNG'!L12&lt;&gt;"",'NHẬP HÀNG'!L12,'DỮ LIỆU FASTMOSS'!E12))</f>
-        <v/>
-      </c>
-      <c r="E12" s="13">
-        <f>IF(OR(A12="",'NHẬP HÀNG'!C12=""),"",'NHẬP HÀNG'!C12+'NHẬP HÀNG'!D12*'NHẬP HÀNG'!E12+'NHẬP HÀNG'!F12+'NHẬP HÀNG'!G12+'NHẬP HÀNG'!H12+'NHẬP HÀNG'!I12)</f>
-        <v/>
-      </c>
-      <c r="F12" s="13">
+      <c r="D12" s="18">
+        <f>IF(A12="","",IF('NHẬP HÀNG'!P12&lt;&gt;"",'NHẬP HÀNG'!P12,'DỮ LIỆU FASTMOSS'!E12))</f>
+        <v/>
+      </c>
+      <c r="E12" s="18">
+        <f>IF(OR(A12="",'NHẬP HÀNG'!C12=""),"",'NHẬP HÀNG'!C12+'NHẬP HÀNG'!W12+'NHẬP HÀNG'!J12+'NHẬP HÀNG'!K12+'NHẬP HÀNG'!L12+'NHẬP HÀNG'!M12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="18">
         <f>IF(OR(A12="",D12=""),"",D12*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="18">
         <f>IF(OR(A12="",D12=""),"",D12*'DỮ LIỆU FASTMOSS'!I12/100)</f>
         <v/>
       </c>
-      <c r="H12" s="13">
+      <c r="H12" s="18">
         <f>IF(A12="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I12" s="13">
+      <c r="I12" s="18">
         <f>IF(OR(A12="",D12=""),"",D12*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J12" s="14">
+      <c r="J12" s="19">
         <f>IF(OR(E12="",D12=""),"",D12-E12-F12-H12-I12)</f>
         <v/>
       </c>
-      <c r="K12" s="15">
+      <c r="K12" s="20">
         <f>IF(J12="","",IFERROR(J12/D12,""))</f>
         <v/>
       </c>
-      <c r="L12" s="13">
+      <c r="L12" s="18">
         <f>IF(J12="","",J12-G12)</f>
         <v/>
       </c>
-      <c r="M12" s="13">
+      <c r="M12" s="18">
         <f>IF(J12="","",J12-D12*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N12" s="14">
+      <c r="N12" s="19">
         <f>IF(OR(E12="",D12=""),"",D12*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H12+(E12-'NHẬP HÀNG'!C12)))</f>
         <v/>
       </c>
-      <c r="O12" s="14">
+      <c r="O12" s="19">
         <f>IF(E12="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E12+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H12)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -2079,7 +2514,7 @@
         <f>IF(OR(NOT(ISNUMBER(O12)),'DỮ LIỆU FASTMOSS'!D12=""),"",IF(O12&lt;'DỮ LIỆU FASTMOSS'!D12,"Thấp hơn mọi đối thủ",IF(O12&lt;='DỮ LIỆU FASTMOSS'!E12,"Dưới hoặc bằng trung vị",IF(O12&lt;='DỮ LIỆU FASTMOSS'!F12,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q12" s="16">
+      <c r="Q12" s="21">
         <f>IF(A12="","",IF(E12="","Chờ nhập hàng",IF(AND(K12&gt;='THAM SỐ'!C6,NOT(P12="Cao hơn mọi đối thủ")),"Làm",IF(J12&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -2097,51 +2532,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B13="","",'DỮ LIỆU FASTMOSS'!B13)</f>
         <v/>
       </c>
-      <c r="D13" s="13">
-        <f>IF(A13="","",IF('NHẬP HÀNG'!L13&lt;&gt;"",'NHẬP HÀNG'!L13,'DỮ LIỆU FASTMOSS'!E13))</f>
-        <v/>
-      </c>
-      <c r="E13" s="13">
-        <f>IF(OR(A13="",'NHẬP HÀNG'!C13=""),"",'NHẬP HÀNG'!C13+'NHẬP HÀNG'!D13*'NHẬP HÀNG'!E13+'NHẬP HÀNG'!F13+'NHẬP HÀNG'!G13+'NHẬP HÀNG'!H13+'NHẬP HÀNG'!I13)</f>
-        <v/>
-      </c>
-      <c r="F13" s="13">
+      <c r="D13" s="18">
+        <f>IF(A13="","",IF('NHẬP HÀNG'!P13&lt;&gt;"",'NHẬP HÀNG'!P13,'DỮ LIỆU FASTMOSS'!E13))</f>
+        <v/>
+      </c>
+      <c r="E13" s="18">
+        <f>IF(OR(A13="",'NHẬP HÀNG'!C13=""),"",'NHẬP HÀNG'!C13+'NHẬP HÀNG'!W13+'NHẬP HÀNG'!J13+'NHẬP HÀNG'!K13+'NHẬP HÀNG'!L13+'NHẬP HÀNG'!M13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="18">
         <f>IF(OR(A13="",D13=""),"",D13*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G13" s="13">
+      <c r="G13" s="18">
         <f>IF(OR(A13="",D13=""),"",D13*'DỮ LIỆU FASTMOSS'!I13/100)</f>
         <v/>
       </c>
-      <c r="H13" s="13">
+      <c r="H13" s="18">
         <f>IF(A13="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I13" s="13">
+      <c r="I13" s="18">
         <f>IF(OR(A13="",D13=""),"",D13*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J13" s="14">
+      <c r="J13" s="19">
         <f>IF(OR(E13="",D13=""),"",D13-E13-F13-H13-I13)</f>
         <v/>
       </c>
-      <c r="K13" s="15">
+      <c r="K13" s="20">
         <f>IF(J13="","",IFERROR(J13/D13,""))</f>
         <v/>
       </c>
-      <c r="L13" s="13">
+      <c r="L13" s="18">
         <f>IF(J13="","",J13-G13)</f>
         <v/>
       </c>
-      <c r="M13" s="13">
+      <c r="M13" s="18">
         <f>IF(J13="","",J13-D13*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N13" s="14">
+      <c r="N13" s="19">
         <f>IF(OR(E13="",D13=""),"",D13*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H13+(E13-'NHẬP HÀNG'!C13)))</f>
         <v/>
       </c>
-      <c r="O13" s="14">
+      <c r="O13" s="19">
         <f>IF(E13="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E13+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H13)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -2149,7 +2584,7 @@
         <f>IF(OR(NOT(ISNUMBER(O13)),'DỮ LIỆU FASTMOSS'!D13=""),"",IF(O13&lt;'DỮ LIỆU FASTMOSS'!D13,"Thấp hơn mọi đối thủ",IF(O13&lt;='DỮ LIỆU FASTMOSS'!E13,"Dưới hoặc bằng trung vị",IF(O13&lt;='DỮ LIỆU FASTMOSS'!F13,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q13" s="16">
+      <c r="Q13" s="21">
         <f>IF(A13="","",IF(E13="","Chờ nhập hàng",IF(AND(K13&gt;='THAM SỐ'!C6,NOT(P13="Cao hơn mọi đối thủ")),"Làm",IF(J13&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -2167,51 +2602,51 @@
         <f>IF('DỮ LIỆU FASTMOSS'!B14="","",'DỮ LIỆU FASTMOSS'!B14)</f>
         <v/>
       </c>
-      <c r="D14" s="13">
-        <f>IF(A14="","",IF('NHẬP HÀNG'!L14&lt;&gt;"",'NHẬP HÀNG'!L14,'DỮ LIỆU FASTMOSS'!E14))</f>
-        <v/>
-      </c>
-      <c r="E14" s="13">
-        <f>IF(OR(A14="",'NHẬP HÀNG'!C14=""),"",'NHẬP HÀNG'!C14+'NHẬP HÀNG'!D14*'NHẬP HÀNG'!E14+'NHẬP HÀNG'!F14+'NHẬP HÀNG'!G14+'NHẬP HÀNG'!H14+'NHẬP HÀNG'!I14)</f>
-        <v/>
-      </c>
-      <c r="F14" s="13">
+      <c r="D14" s="18">
+        <f>IF(A14="","",IF('NHẬP HÀNG'!P14&lt;&gt;"",'NHẬP HÀNG'!P14,'DỮ LIỆU FASTMOSS'!E14))</f>
+        <v/>
+      </c>
+      <c r="E14" s="18">
+        <f>IF(OR(A14="",'NHẬP HÀNG'!C14=""),"",'NHẬP HÀNG'!C14+'NHẬP HÀNG'!W14+'NHẬP HÀNG'!J14+'NHẬP HÀNG'!K14+'NHẬP HÀNG'!L14+'NHẬP HÀNG'!M14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="18">
         <f>IF(OR(A14="",D14=""),"",D14*(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19))+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18))</f>
         <v/>
       </c>
-      <c r="G14" s="13">
+      <c r="G14" s="18">
         <f>IF(OR(A14="",D14=""),"",D14*'DỮ LIỆU FASTMOSS'!I14/100)</f>
         <v/>
       </c>
-      <c r="H14" s="13">
+      <c r="H14" s="18">
         <f>IF(A14="","",IFERROR('THAM SỐ'!C10/'THAM SỐ'!C11,0)+'THAM SỐ'!C12+'THAM SỐ'!C9)</f>
         <v/>
       </c>
-      <c r="I14" s="13">
+      <c r="I14" s="18">
         <f>IF(OR(A14="",D14=""),"",D14*'THAM SỐ'!C8)</f>
         <v/>
       </c>
-      <c r="J14" s="14">
+      <c r="J14" s="19">
         <f>IF(OR(E14="",D14=""),"",D14-E14-F14-H14-I14)</f>
         <v/>
       </c>
-      <c r="K14" s="15">
+      <c r="K14" s="20">
         <f>IF(J14="","",IFERROR(J14/D14,""))</f>
         <v/>
       </c>
-      <c r="L14" s="13">
+      <c r="L14" s="18">
         <f>IF(J14="","",J14-G14)</f>
         <v/>
       </c>
-      <c r="M14" s="13">
+      <c r="M14" s="18">
         <f>IF(J14="","",J14-D14*'THAM SỐ'!C7)</f>
         <v/>
       </c>
-      <c r="N14" s="14">
+      <c r="N14" s="19">
         <f>IF(OR(E14="",D14=""),"",D14*(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)-(IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H14+(E14-'NHẬP HÀNG'!C14)))</f>
         <v/>
       </c>
-      <c r="O14" s="14">
+      <c r="O14" s="19">
         <f>IF(E14="","",IF((IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)+'THAM SỐ'!C8+'THAM SỐ'!C6)&gt;=1,"Không khả thi",(E14+IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$18,'THAM SỐ'!$D$18)+H14)/(1-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$16,'THAM SỐ'!$D$16)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$17,'THAM SỐ'!$D$17)-IF('THAM SỐ'!$C$4="VN",'THAM SỐ'!$C$19,'THAM SỐ'!$D$19)-'THAM SỐ'!C8-'THAM SỐ'!C6)))</f>
         <v/>
       </c>
@@ -2219,7 +2654,7 @@
         <f>IF(OR(NOT(ISNUMBER(O14)),'DỮ LIỆU FASTMOSS'!D14=""),"",IF(O14&lt;'DỮ LIỆU FASTMOSS'!D14,"Thấp hơn mọi đối thủ",IF(O14&lt;='DỮ LIỆU FASTMOSS'!E14,"Dưới hoặc bằng trung vị",IF(O14&lt;='DỮ LIỆU FASTMOSS'!F14,"Trên trung vị, trong vùng giá","Cao hơn mọi đối thủ"))))</f>
         <v/>
       </c>
-      <c r="Q14" s="16">
+      <c r="Q14" s="21">
         <f>IF(A14="","",IF(E14="","Chờ nhập hàng",IF(AND(K14&gt;='THAM SỐ'!C6,NOT(P14="Cao hơn mọi đối thủ")),"Làm",IF(J14&gt;0,"Cân nhắc","Bỏ"))))</f>
         <v/>
       </c>
@@ -2228,6 +2663,501 @@
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Đọc kết quả: Làm = lời đạt biên mong muốn và giá đề xuất không cao hơn mọi đối thủ. Cân nhắc = có lời nhưng mỏng hoặc giá cao. Bỏ = lỗ. Nếu nhà cung cấp báo cao hơn Giá nhập tối đa thì đàm phán hoặc bỏ.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>BẢNG CƯỚC ĐI US VÀ CANADA (VND)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Mentor cập nhật khi hãng đổi giá. Ô vàng là số cước, sheet NHẬP HÀNG tự tra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>VPS EXPRESS (hàng thường 8 đến 10 ngày, hàng khó 10 đến 14 ngày)</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="inlineStr">
+        <is>
+          <t>AM EXPRESS (10 đến 14 ngày, giao tận nhà, bao thuế nhập khẩu, hiệu lực 01/10 đến 31/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Trọng lượng (kg)</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Cước (VND)</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Trọng lượng (kg)</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Cước (VND)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>1810000</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>1025000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>2120000</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>1225000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>2530000</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>1425000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>2830000</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>1625000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>3240000</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>1825000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>3550000</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>2025000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>3910000</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>2225000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>4170000</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>2425000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>4370000</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>2625000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>4710000</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>2825000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>4850000</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>3200000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>5130000</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>3400000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>5280000</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>5380000</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>3800000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>5480000</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>4000000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>5600000</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>4200000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>5700000</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>4400000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>5850000</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>4600000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>5950000</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>4800000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="F25" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>5100000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>Từ 21kg</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>(mỗi kg)</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>5400000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Giá mỗi kg</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>269000</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>5700000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="F28" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>6000000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="F29" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>6300000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="F30" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G30" s="8" t="n">
+        <v>6600000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="F31" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>6900000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="F32" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="G32" s="8" t="n">
+        <v>7200000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="F33" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>7500000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="F34" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>7800000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Giá mỗi kg từ 21kg</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Cách tính cước: lấy lớn hơn giữa cân nặng thật và cân nặng quy đổi (dài x rộng x cao cm chia 5000), nhân số lượng, làm tròn lên: VPS tròn 1 kg, AM tròn 0,5 kg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>VPS: giá chưa gồm VAT (cộng 8% nếu lấy hóa đơn), chưa gồm bảo hiểm 10 đến 20% giá trị hàng. Miễn phí xử lý, đóng thùng, dán nhãn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>AM: giao tận nhà, bao thuế nhập khẩu. VPS không ghi rõ thuế nhập khẩu, cần hỏi lại trước khi so giá.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Công thức quy đổi của AM chưa ghi trong báo giá, sheet tạm dùng /5000 giống VPS. Hỏi lại AM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Hai hãng khác điều kiện (thuế, bảo hiểm, thời gian), nên cước rẻ nhất chưa chắc là lựa chọn tốt nhất.</t>
         </is>
       </c>
     </row>

</xml_diff>